<commit_message>
Update XC24R TRIM JIG 디버깅 LIST.xlsx
</commit_message>
<xml_diff>
--- a/X-Series/XD12R/Jig/XCR_XDR/XC24RV_XD12RV/HW/XC24R TRIM JIG 디버깅 LIST.xlsx
+++ b/X-Series/XD12R/Jig/XCR_XDR/XC24RV_XD12RV/HW/XC24R TRIM JIG 디버깅 LIST.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\working\01_Project\FW\X-Series\XD12R\Jig\XCR_XDR\XC24RV_XD12RV\HW\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B234826F-B144-4005-9B25-C7503523198E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF5CD5D3-A273-4167-9839-3CC6139FD87E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43080" yWindow="2160" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{32538B79-DC4A-44A8-A8C4-6C0535803166}"/>
+    <workbookView xWindow="43080" yWindow="2160" windowWidth="29040" windowHeight="15720" xr2:uid="{32538B79-DC4A-44A8-A8C4-6C0535803166}"/>
   </bookViews>
   <sheets>
     <sheet name="07_06 1일차" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="61">
   <si>
     <t>수정</t>
     <phoneticPr fontId="2" type="noConversion"/>
@@ -260,6 +260,38 @@
   </si>
   <si>
     <t>외장 ADC</t>
+  </si>
+  <si>
+    <t>-</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Pin. 2 (VSS)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Pin. 5 (Dio)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Pin. 6 (SVI)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Pin. 16 (VSS)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Pin. 15 (VSS)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Pin. 14 (Ddio)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Pin. 5 (Dio) 버퍼 전원</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -311,7 +343,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="26">
     <border>
       <left/>
       <right/>
@@ -493,13 +525,188 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -536,53 +743,116 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -881,9 +1151,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>16</xdr:col>
-      <xdr:colOff>197237</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>609773</xdr:rowOff>
+      <xdr:colOff>200412</xdr:colOff>
+      <xdr:row>8</xdr:row>
+      <xdr:rowOff>57323</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -927,7 +1197,7 @@
       <xdr:col>5</xdr:col>
       <xdr:colOff>1488039</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>962025</xdr:rowOff>
+      <xdr:rowOff>958850</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -952,6 +1222,94 @@
         <a:xfrm>
           <a:off x="6543675" y="1076325"/>
           <a:ext cx="1488039" cy="962025"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>1511300</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>735552</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="그림 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{86093592-393E-487B-93BC-FD5C54AFEF0E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6781800" y="3152776"/>
+          <a:ext cx="1514475" cy="738726"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>1</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>388385</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="그림 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{759C0CC8-BDF0-D7E1-A76E-FA5EBF92DDCA}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6781801" y="2095501"/>
+          <a:ext cx="1524000" cy="394734"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1280,7 +1638,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{084D8CD6-32BA-42AD-869C-9A6DD7BC206C}">
-  <dimension ref="B2:O31"/>
+  <dimension ref="B1:O31"/>
   <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="16" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="2.81640625" style="1" customWidth="1"/>
@@ -1300,54 +1658,59 @@
     <col min="18" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:15" x14ac:dyDescent="0.45">
-      <c r="B2" s="12" t="s">
+    <row r="1" spans="2:15" ht="16.5" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="2" spans="2:15" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B2" s="43" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="E2" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="12" t="s">
+      <c r="F2" s="37" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="3" spans="2:15" ht="53" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="44" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="C3" s="39" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
+      <c r="E3" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="F3" s="35"/>
     </row>
     <row r="4" spans="2:15" ht="143" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="45" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="40" t="s">
         <v>21</v>
       </c>
       <c r="D4" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
+      <c r="E4" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="F4" s="28"/>
     </row>
     <row r="5" spans="2:15" ht="83" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B5" s="12" t="s">
+      <c r="B5" s="45" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="41" t="s">
         <v>22</v>
       </c>
       <c r="D5" s="10" t="s">
@@ -1356,13 +1719,13 @@
       <c r="E5" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="F5" s="10"/>
+      <c r="F5" s="28"/>
     </row>
     <row r="6" spans="2:15" ht="96" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B6" s="12" t="s">
+      <c r="B6" s="45" t="s">
         <v>25</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="41" t="s">
         <v>22</v>
       </c>
       <c r="D6" s="10" t="s">
@@ -1371,22 +1734,22 @@
       <c r="E6" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="F6" s="10"/>
-    </row>
-    <row r="7" spans="2:15" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B7" s="12" t="s">
+      <c r="F6" s="28"/>
+    </row>
+    <row r="7" spans="2:15" ht="80" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B7" s="46" t="s">
         <v>28</v>
       </c>
-      <c r="C7" s="10" t="s">
+      <c r="C7" s="42" t="s">
         <v>29</v>
       </c>
-      <c r="D7" s="10" t="s">
+      <c r="D7" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="E7" s="10" t="s">
+      <c r="E7" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="F7" s="10"/>
+      <c r="F7" s="2"/>
     </row>
     <row r="14" spans="2:15" x14ac:dyDescent="0.45">
       <c r="O14" s="3"/>
@@ -1411,7 +1774,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{088542B5-32EE-4CC9-976A-EFFC98E2A0B2}">
-  <dimension ref="B2:O31"/>
+  <dimension ref="B1:O31"/>
   <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="16" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="2.81640625" style="1" customWidth="1"/>
@@ -1431,80 +1794,85 @@
     <col min="18" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:15" x14ac:dyDescent="0.45">
-      <c r="B2" s="12" t="s">
+    <row r="1" spans="2:15" ht="16.5" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="2" spans="2:15" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B2" s="43" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="C2" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="D2" s="36" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="12" t="s">
+      <c r="E2" s="36" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="12" t="s">
+      <c r="F2" s="37" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="3" spans="2:15" ht="53" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B3" s="12" t="s">
+      <c r="B3" s="44" t="s">
         <v>33</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="C3" s="48" t="s">
         <v>49</v>
       </c>
-      <c r="D3" s="10" t="s">
+      <c r="D3" s="33" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
+      <c r="E3" s="34" t="s">
+        <v>53</v>
+      </c>
+      <c r="F3" s="35"/>
     </row>
     <row r="4" spans="2:15" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="45" t="s">
         <v>37</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="40" t="s">
         <v>50</v>
       </c>
       <c r="D4" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
-    </row>
-    <row r="5" spans="2:15" ht="83" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B5" s="12" t="s">
+      <c r="E4" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="F4" s="28"/>
+    </row>
+    <row r="5" spans="2:15" ht="35" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B5" s="45" t="s">
         <v>38</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C5" s="41" t="s">
         <v>51</v>
       </c>
       <c r="D5" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
-    </row>
-    <row r="6" spans="2:15" ht="96" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B6" s="12" t="s">
+      <c r="E5" s="19" t="s">
+        <v>53</v>
+      </c>
+      <c r="F5" s="28"/>
+    </row>
+    <row r="6" spans="2:15" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B6" s="46" t="s">
         <v>48</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="42" t="s">
         <v>52</v>
       </c>
-      <c r="D6" s="10"/>
-      <c r="E6" s="11"/>
-      <c r="F6" s="10"/>
-    </row>
-    <row r="7" spans="2:15" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B7" s="12"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
-      <c r="E7" s="10"/>
-      <c r="F7" s="10"/>
-    </row>
+      <c r="D6" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="47" t="s">
+        <v>53</v>
+      </c>
+      <c r="F6" s="2"/>
+    </row>
+    <row r="7" spans="2:15" ht="16" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="14" spans="2:15" x14ac:dyDescent="0.45">
       <c r="O14" s="3"/>
     </row>
@@ -1548,172 +1916,203 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C2B1110-480D-43CA-ADDF-C33DF1BCB179}">
-  <dimension ref="B1:G13"/>
+  <dimension ref="B1:H13"/>
   <sheetFormatPr defaultRowHeight="16" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="2.6328125" customWidth="1"/>
-    <col min="2" max="3" width="26" customWidth="1"/>
-    <col min="5" max="6" width="23.90625" customWidth="1"/>
-    <col min="7" max="7" width="17.36328125" customWidth="1"/>
+    <col min="2" max="4" width="26" customWidth="1"/>
+    <col min="6" max="7" width="23.90625" customWidth="1"/>
+    <col min="8" max="8" width="17.36328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.5"/>
-    <row r="2" spans="2:7" x14ac:dyDescent="0.45">
-      <c r="B2" s="14" t="s">
+    <row r="1" spans="2:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="2" spans="2:8" x14ac:dyDescent="0.45">
+      <c r="B2" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="15"/>
-      <c r="E2" s="14" t="s">
+      <c r="C2" s="31"/>
+      <c r="D2" s="32"/>
+      <c r="F2" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="F2" s="17"/>
-      <c r="G2" s="15"/>
-    </row>
-    <row r="3" spans="2:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="G2" s="24"/>
+      <c r="H2" s="21"/>
+    </row>
+    <row r="3" spans="2:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B3" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="D3" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="F3" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="F3" s="23" t="s">
+      <c r="G3" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="G3" s="24" t="s">
+      <c r="H3" s="2" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="4" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="4" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B4" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="D4" s="9" t="s">
+        <v>54</v>
+      </c>
+      <c r="F4" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="F4" s="21" t="s">
+      <c r="G4" s="17" t="s">
         <v>32</v>
       </c>
-      <c r="G4" s="22" t="s">
+      <c r="H4" s="22" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="5" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="19" t="s">
+      <c r="D5" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="F5" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="F5" s="16" t="s">
+      <c r="G5" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="G5" s="18"/>
-    </row>
-    <row r="6" spans="2:7" x14ac:dyDescent="0.45">
+      <c r="H5" s="23"/>
+    </row>
+    <row r="6" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B6" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="E6" s="19" t="s">
+      <c r="D6" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="F6" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="F6" s="16" t="s">
+      <c r="G6" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="G6" s="25" t="s">
+      <c r="H6" s="14" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="7" spans="2:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+    <row r="7" spans="2:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B7" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="E7" s="26" t="s">
+      <c r="D7" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="F7" s="25" t="s">
         <v>41</v>
       </c>
-      <c r="F7" s="27"/>
-      <c r="G7" s="20" t="s">
+      <c r="G7" s="26"/>
+      <c r="H7" s="16" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="2:7" x14ac:dyDescent="0.45">
+    <row r="8" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B8" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="E8" s="13"/>
-      <c r="F8" s="13"/>
-      <c r="G8" s="13"/>
-    </row>
-    <row r="9" spans="2:7" x14ac:dyDescent="0.45">
+      <c r="D8" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="F8" s="12"/>
+      <c r="G8" s="12"/>
+      <c r="H8" s="12"/>
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B9" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="E9" s="13"/>
-      <c r="F9" s="13"/>
-      <c r="G9" s="13"/>
-    </row>
-    <row r="10" spans="2:7" x14ac:dyDescent="0.45">
+      <c r="D9" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="F9" s="12"/>
+      <c r="G9" s="12"/>
+      <c r="H9" s="12"/>
+    </row>
+    <row r="10" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B10" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="E10" s="13"/>
-      <c r="F10" s="13"/>
-      <c r="G10" s="13"/>
-    </row>
-    <row r="11" spans="2:7" x14ac:dyDescent="0.45">
+      <c r="D10" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="F10" s="12"/>
+      <c r="G10" s="12"/>
+      <c r="H10" s="12"/>
+    </row>
+    <row r="11" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B11" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="E11" s="13"/>
-      <c r="F11" s="13"/>
-      <c r="G11" s="13"/>
-    </row>
-    <row r="12" spans="2:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="D11" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="F11" s="12"/>
+      <c r="G11" s="12"/>
+      <c r="H11" s="12"/>
+    </row>
+    <row r="12" spans="2:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B12" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="C12" s="7" t="s">
+      <c r="C12" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="E12" s="13"/>
-      <c r="F12" s="13"/>
-      <c r="G12" s="13"/>
-    </row>
-    <row r="13" spans="2:7" x14ac:dyDescent="0.45">
-      <c r="G13" s="13"/>
+      <c r="D12" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="F12" s="12"/>
+      <c r="G12" s="12"/>
+      <c r="H12" s="12"/>
+    </row>
+    <row r="13" spans="2:8" x14ac:dyDescent="0.45">
+      <c r="H13" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="G4:G5"/>
-    <mergeCell ref="E2:G2"/>
-    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="B2:D2"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
minor update, 자료 업뎃
</commit_message>
<xml_diff>
--- a/X-Series/XD12R/Jig/XCR_XDR/XC24RV_XD12RV/HW/XC24R TRIM JIG 디버깅 LIST.xlsx
+++ b/X-Series/XD12R/Jig/XCR_XDR/XC24RV_XD12RV/HW/XC24R TRIM JIG 디버깅 LIST.xlsx
@@ -8,16 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\working\01_Project\FW\X-Series\XD12R\Jig\XCR_XDR\XC24RV_XD12RV\HW\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF5CD5D3-A273-4167-9839-3CC6139FD87E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{037B954C-9710-45A3-AAFA-6902F0019703}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="43080" yWindow="2160" windowWidth="29040" windowHeight="15720" xr2:uid="{32538B79-DC4A-44A8-A8C4-6C0535803166}"/>
+    <workbookView xWindow="71880" yWindow="2160" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{32538B79-DC4A-44A8-A8C4-6C0535803166}"/>
   </bookViews>
   <sheets>
     <sheet name="07_06 1일차" sheetId="1" r:id="rId1"/>
     <sheet name="07_07 2일차" sheetId="5" r:id="rId2"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId3"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId4"/>
-    <sheet name="스위치 설정 가이드" sheetId="4" r:id="rId5"/>
+    <sheet name="07_08 3일차" sheetId="2" r:id="rId3"/>
+    <sheet name="07_09 4일차" sheetId="7" r:id="rId4"/>
+    <sheet name="VDD 3V3" sheetId="3" r:id="rId5"/>
+    <sheet name="XDR 스위치" sheetId="4" r:id="rId6"/>
+    <sheet name="XCR 스위치" sheetId="6" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -43,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="147">
   <si>
     <t>수정</t>
     <phoneticPr fontId="2" type="noConversion"/>
@@ -291,6 +293,342 @@
   </si>
   <si>
     <t>Pin. 5 (Dio) 버퍼 전원</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>IC No.</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>#1-1</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>#1-2</t>
+  </si>
+  <si>
+    <t>#1-3</t>
+  </si>
+  <si>
+    <t>#1-4</t>
+  </si>
+  <si>
+    <t>#1-5</t>
+  </si>
+  <si>
+    <t>#2</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>#3</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>#4</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>#5</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>CH2</t>
+  </si>
+  <si>
+    <t>CH3</t>
+  </si>
+  <si>
+    <t>CH4</t>
+  </si>
+  <si>
+    <t>CH5</t>
+  </si>
+  <si>
+    <t>CH6</t>
+  </si>
+  <si>
+    <t>CH7</t>
+  </si>
+  <si>
+    <t>CH8</t>
+  </si>
+  <si>
+    <t>CH9</t>
+  </si>
+  <si>
+    <t>CH10</t>
+  </si>
+  <si>
+    <t>CH11</t>
+  </si>
+  <si>
+    <t>CH12</t>
+  </si>
+  <si>
+    <t>비고</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>동일 IC
+5회 반복</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>초기 시행 결과 (#1-1)
+대비 변화량</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>NG</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>주파수 OSC [MHz]</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>CH1 [mA]</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>변화량 #1-2</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>변화량 #1-3</t>
+  </si>
+  <si>
+    <t>변화량 #1-4</t>
+  </si>
+  <si>
+    <t>변화량 #1-5</t>
+  </si>
+  <si>
+    <t>XD 주파수 Measure
+(ZIF Socket)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>XD Iout Measure
+(ZIF Socket)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>XD Icc measure
+(ZIF Socket)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt; PCB 전원층&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt; PCB Top View&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt; Daisy 검토용 ZIF Socket &gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt; 신뢰성 후 측정용 ZIF Socket &gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>스위치 셋팅 for XD controlled by XCR (미검토)</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>SW4 (Piano)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>all on</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>SPI, VSYNC, FLLSYNC, MCLK</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>SW5 (Piano)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>all off</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>SW7 (Piano)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Pin. 2 (TEST1)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>J57</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>off</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Pin. 3 (FLLSYNC)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>SW8 (Piano)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>SW10 (Piano)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>SW12 (Piano)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Pin. 11 (nINT_LD)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Pin. 13 (MCLK)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Pin. 22 (GND)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>SW11 (Piano)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>1, 3 on</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Pin. 35 (L_G1), Pin. 36 (H_G1)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>SW9 (Piano)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>1, 4 on</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Pin. 38 (LDOO), Pin. 40 (TESTA)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>SW6 (Piano)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Pin. 56 (GND)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Right</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>스위치 셋팅 for XCR ES0 (미검토)</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>스위치 셋팅 for XCR ES0 Trim (미검토)</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>XC VSYNC</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>XC FLLSYNC</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>XC MCLK</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt; 임시 방편 &gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>XC SPI</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Piano 스위치
+(MCU, FPGA 구분)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>전원 Source 변경 필요
+VDD 3V3이 PCB 전원층에 
+Plane 형태로 넓게 결합되어 있어패턴 커팅 등의 수정이 불가함
+임시 방편 적용 필요
+(VDD 3V3 시트 참조)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>SW37</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>VDD Selection</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>보드 간 편차</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Board No</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>#1</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Vref [V]</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>XD 주파수, Vref전압, 출력 전류</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>AVG</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>평균값 대비 편차</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>편차 #1</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>편차 #2</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>편차 #3</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>편차 #4</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -298,7 +636,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="176" formatCode="0.000"/>
+  </numFmts>
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color theme="1"/>
@@ -328,8 +669,40 @@
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="2" tint="-9.9978637043366805E-2"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="2" tint="-9.9978637043366805E-2"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -342,8 +715,26 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="26">
+  <borders count="51">
     <border>
       <left/>
       <right/>
@@ -700,13 +1091,331 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="153">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -734,9 +1443,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -767,27 +1473,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -795,15 +1480,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -854,8 +1530,354 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="3" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="1" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="1" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="1" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="1" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="1" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="1" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="1" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="1" fillId="0" borderId="33" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="3" borderId="26" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="3" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="41" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="38" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="44" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="46" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="47" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="43" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="1" fillId="0" borderId="45" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="1" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="1" fillId="0" borderId="50" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="1" fillId="5" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="1" fillId="5" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="1" fillId="5" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="30" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="31" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="1" fillId="0" borderId="32" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="백분율" xfId="1" builtinId="5"/>
     <cellStyle name="표준" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1321,6 +2343,1641 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>56031</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>33618</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>1</xdr:colOff>
+      <xdr:row>4</xdr:row>
+      <xdr:rowOff>817357</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="그림 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D15E0C8B-8A8D-11E9-FB2E-1B09EFE7F91E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7171766" y="2151530"/>
+          <a:ext cx="1467970" cy="783739"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>19237</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>11206</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>1504764</xdr:colOff>
+      <xdr:row>9</xdr:row>
+      <xdr:rowOff>2351</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="그림 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C84C41A9-A28C-4EFD-94AA-CF48D5B79A05}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7134972" y="3339353"/>
+          <a:ext cx="1485527" cy="932439"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>25590</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>25503</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="30" name="그림 29">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AEF6A19A-6017-4613-8EDA-9FD73F065A6E}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="182217" y="5449957"/>
+          <a:ext cx="3706243" cy="2016504"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>398933</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>142218</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="29" name="그림 28">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{30A33DFD-B7EF-4553-9621-DE7B6B14F125}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch/>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4463143" y="5578929"/>
+          <a:ext cx="11420719" cy="1775075"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>100853</xdr:rowOff>
+    </xdr:to>
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="24" name="그룹 23">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{54F4CB24-AD84-315D-633B-AC1074F598BC}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
+        <a:xfrm>
+          <a:off x="6234545" y="536864"/>
+          <a:ext cx="5455228" cy="4468209"/>
+          <a:chOff x="6230471" y="549088"/>
+          <a:chExt cx="5364141" cy="4276629"/>
+        </a:xfrm>
+      </xdr:grpSpPr>
+      <xdr:pic>
+        <xdr:nvPicPr>
+          <xdr:cNvPr id="6" name="그림 5">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F3B863AC-ED72-4DF7-9FD5-ED4F6476E8CC}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvPicPr>
+            <a:picLocks noChangeAspect="1"/>
+          </xdr:cNvPicPr>
+        </xdr:nvPicPr>
+        <xdr:blipFill>
+          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
+          <a:stretch>
+            <a:fillRect/>
+          </a:stretch>
+        </xdr:blipFill>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="6230471" y="549088"/>
+            <a:ext cx="5364141" cy="4276629"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln>
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+      </xdr:pic>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="11" name="화살표: 오른쪽 10">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C570FE76-60B1-4EB1-9011-F1294C264745}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="7356290" y="1479737"/>
+            <a:ext cx="655918" cy="227106"/>
+          </a:xfrm>
+          <a:prstGeom prst="rightArrow">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="FFFF00"/>
+          </a:solidFill>
+          <a:ln>
+            <a:solidFill>
+              <a:srgbClr val="FFFF00"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:endParaRPr lang="ko-KR" altLang="en-US" sz="1100"/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="12" name="화살표: 오른쪽 11">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0E7ADD60-589A-46FE-8659-7E644B46A507}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm rot="5400000">
+            <a:off x="6767140" y="2948923"/>
+            <a:ext cx="670299" cy="231775"/>
+          </a:xfrm>
+          <a:prstGeom prst="rightArrow">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="FFFF00"/>
+          </a:solidFill>
+          <a:ln>
+            <a:solidFill>
+              <a:srgbClr val="FFFF00"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:endParaRPr lang="ko-KR" altLang="en-US" sz="1100"/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="13" name="화살표: 오른쪽 12">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CC5A4013-2246-45C6-AAB0-2B498823F0D9}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm rot="5400000">
+            <a:off x="8571381" y="2969560"/>
+            <a:ext cx="673474" cy="225425"/>
+          </a:xfrm>
+          <a:prstGeom prst="rightArrow">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="FFFF00"/>
+          </a:solidFill>
+          <a:ln>
+            <a:solidFill>
+              <a:srgbClr val="FFFF00"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:endParaRPr lang="ko-KR" altLang="en-US" sz="1100"/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="14" name="화살표: 오른쪽 13">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5CEB0226-43E7-4FF7-8F79-EA5CC63B6EC3}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm rot="5400000">
+            <a:off x="10367684" y="2940985"/>
+            <a:ext cx="673474" cy="231775"/>
+          </a:xfrm>
+          <a:prstGeom prst="rightArrow">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="FFFF00"/>
+          </a:solidFill>
+          <a:ln>
+            <a:solidFill>
+              <a:srgbClr val="FFFF00"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:endParaRPr lang="ko-KR" altLang="en-US" sz="1100"/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="15" name="TextBox 14">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{920D3F7C-AF1A-55EA-5B3D-A9064E85947E}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr txBox="1"/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="6840070" y="1806949"/>
+            <a:ext cx="4181475" cy="790986"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:schemeClr val="bg1"/>
+          </a:solidFill>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="ctr">
+            <a:spAutoFit/>
+          </a:bodyPr>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr"/>
+            <a:r>
+              <a:rPr lang="en-US" altLang="ko-KR" sz="1050">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>VDD 3V3</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="ko-KR" altLang="en-US" sz="1050">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>전원이 </a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" altLang="ko-KR" sz="1050">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>PCB </a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="ko-KR" altLang="en-US" sz="1050">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>전원층에</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-US" altLang="ko-KR" sz="1050">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+            </a:endParaRPr>
+          </a:p>
+          <a:p>
+            <a:pPr algn="ctr"/>
+            <a:r>
+              <a:rPr lang="en-US" altLang="ko-KR" sz="1050">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>Plane </a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="ko-KR" altLang="en-US" sz="1050">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>형태로 구성되어 있음</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" altLang="ko-KR" sz="1050">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>.</a:t>
+            </a:r>
+          </a:p>
+          <a:p>
+            <a:pPr algn="ctr"/>
+            <a:r>
+              <a:rPr lang="ko-KR" altLang="en-US" sz="1050">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>수정이 불가함</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" altLang="ko-KR" sz="1050">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>.</a:t>
+            </a:r>
+            <a:endParaRPr lang="ko-KR" altLang="en-US" sz="1050">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="17" name="직사각형 16">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1458B99D-0687-4B7F-8BB0-7B5505225743}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="6278096" y="711013"/>
+            <a:ext cx="795617" cy="220756"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln w="76200">
+            <a:solidFill>
+              <a:srgbClr val="FFFF00"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:endParaRPr lang="ko-KR" altLang="en-US" sz="1100"/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+    </xdr:grpSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>10</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>142501</xdr:rowOff>
+    </xdr:to>
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="23" name="그룹 22">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EC825EC9-1C90-ECB6-FB84-9D4B2BD5CA77}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
+        <a:xfrm>
+          <a:off x="173182" y="536874"/>
+          <a:ext cx="5455227" cy="4509847"/>
+          <a:chOff x="179294" y="549098"/>
+          <a:chExt cx="5367316" cy="4276651"/>
+        </a:xfrm>
+      </xdr:grpSpPr>
+      <xdr:pic>
+        <xdr:nvPicPr>
+          <xdr:cNvPr id="4" name="그림 3">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D146EDC4-BC60-48D0-B211-DE5C8504210A}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvPicPr>
+            <a:picLocks noChangeAspect="1"/>
+          </xdr:cNvPicPr>
+        </xdr:nvPicPr>
+        <xdr:blipFill>
+          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
+          <a:stretch>
+            <a:fillRect/>
+          </a:stretch>
+        </xdr:blipFill>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="179294" y="549098"/>
+            <a:ext cx="5367316" cy="4276651"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:ln>
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+      </xdr:pic>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="7" name="화살표: 오른쪽 6">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{91033732-8567-BC95-D6EF-AD35AB87E660}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="1305112" y="1470212"/>
+            <a:ext cx="655917" cy="227106"/>
+          </a:xfrm>
+          <a:prstGeom prst="rightArrow">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="FFFF00"/>
+          </a:solidFill>
+          <a:ln>
+            <a:solidFill>
+              <a:srgbClr val="FFFF00"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:endParaRPr lang="ko-KR" altLang="en-US" sz="1100"/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="8" name="화살표: 오른쪽 7">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4DD16CFF-3161-477C-B023-803A0BCCCA73}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm rot="5400000">
+            <a:off x="714375" y="2940985"/>
+            <a:ext cx="673474" cy="231775"/>
+          </a:xfrm>
+          <a:prstGeom prst="rightArrow">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="FFFF00"/>
+          </a:solidFill>
+          <a:ln>
+            <a:solidFill>
+              <a:srgbClr val="FFFF00"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:endParaRPr lang="ko-KR" altLang="en-US" sz="1100"/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="9" name="화살표: 오른쪽 8">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{46ED1AAC-F1A9-467B-9F46-56814B138FC2}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm rot="5400000">
+            <a:off x="2518615" y="2961623"/>
+            <a:ext cx="676649" cy="225425"/>
+          </a:xfrm>
+          <a:prstGeom prst="rightArrow">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="FFFF00"/>
+          </a:solidFill>
+          <a:ln>
+            <a:solidFill>
+              <a:srgbClr val="FFFF00"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:endParaRPr lang="ko-KR" altLang="en-US" sz="1100"/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="10" name="화살표: 오른쪽 9">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7445C874-576E-4366-AAC5-6E3F82019B3C}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm rot="5400000">
+            <a:off x="4318093" y="2929873"/>
+            <a:ext cx="670299" cy="231775"/>
+          </a:xfrm>
+          <a:prstGeom prst="rightArrow">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:srgbClr val="FFFF00"/>
+          </a:solidFill>
+          <a:ln>
+            <a:solidFill>
+              <a:srgbClr val="FFFF00"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:endParaRPr lang="ko-KR" altLang="en-US" sz="1100"/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="16" name="직사각형 15">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C0D692EC-4436-3117-E2C2-E9BA5B0F9CCC}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="204694" y="720538"/>
+            <a:ext cx="789268" cy="220756"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+          <a:ln w="76200">
+            <a:solidFill>
+              <a:srgbClr val="FFFF00"/>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="l"/>
+            <a:endParaRPr lang="ko-KR" altLang="en-US" sz="1100"/>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="18" name="TextBox 17">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D81EA42F-D7FE-24E5-B13E-B414B6C17BA4}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr txBox="1"/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="1332846" y="1475519"/>
+            <a:ext cx="579058" cy="231937"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:noFill/>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:lnRef>
+          <a:fillRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:scrgbClr r="0" g="0" b="0"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="tx1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
+            <a:spAutoFit/>
+          </a:bodyPr>
+          <a:lstStyle/>
+          <a:p>
+            <a:r>
+              <a:rPr lang="en-US" altLang="ko-KR" sz="900">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>VDD 3V3</a:t>
+            </a:r>
+            <a:endParaRPr lang="ko-KR" altLang="en-US" sz="900">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+    </xdr:grpSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>39787</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>65645</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>173122</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>164483</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="25" name="화살표: 오른쪽 24">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00DFF17F-1DD9-4642-9B34-EF463A57383D}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm rot="5400000">
+          <a:off x="752775" y="5597744"/>
+          <a:ext cx="297620" cy="133335"/>
+        </a:xfrm>
+        <a:prstGeom prst="rightArrow">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFF00"/>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="ko-KR" altLang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>575527</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>118108</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>95949</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>8386</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="26" name="화살표: 오른쪽 25">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{62245EA9-82F4-48A0-92F0-3C228729D3AE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm rot="5400000">
+          <a:off x="4970882" y="5645319"/>
+          <a:ext cx="287843" cy="133335"/>
+        </a:xfrm>
+        <a:prstGeom prst="rightArrow">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFF00"/>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="ko-KR" altLang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>235941</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>104720</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>369276</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>187431</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="27" name="화살표: 오른쪽 26">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3D1DA084-249E-45A1-814C-E9E20001AAFD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm rot="5400000">
+          <a:off x="8924862" y="5628756"/>
+          <a:ext cx="281493" cy="133335"/>
+        </a:xfrm>
+        <a:prstGeom prst="rightArrow">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFF00"/>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="ko-KR" altLang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>492701</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>113003</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>13123</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>189364</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="28" name="화살표: 오른쪽 27">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D95910E7-AEF8-4111-AC7A-0EA5419149B0}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm rot="5400000">
+          <a:off x="12862275" y="5633864"/>
+          <a:ext cx="275143" cy="133335"/>
+        </a:xfrm>
+        <a:prstGeom prst="rightArrow">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFF00"/>
+        </a:solidFill>
+        <a:ln>
+          <a:solidFill>
+            <a:schemeClr val="tx1"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="ko-KR" altLang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>588065</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>132532</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>573449</xdr:colOff>
+      <xdr:row>7</xdr:row>
+      <xdr:rowOff>167870</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="31" name="TextBox 30">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C58BF632-7C20-42E4-B88B-BD8188AB44D9}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="10841935" y="1466032"/>
+          <a:ext cx="598297" cy="234121"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
+          <a:noAutofit/>
+        </a:bodyPr>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="en-US" altLang="ko-KR" sz="900">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>VDD 3V3</a:t>
+          </a:r>
+          <a:endParaRPr lang="ko-KR" altLang="en-US" sz="900">
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+          </a:endParaRPr>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>11211</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>44827</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>11207</xdr:colOff>
+      <xdr:row>57</xdr:row>
+      <xdr:rowOff>46786</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="그림 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{442794D8-A164-F0AB-F269-559345620C5C}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="190505" y="8348386"/>
+          <a:ext cx="3630702" cy="3632665"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>493059</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>168089</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>219261</xdr:colOff>
+      <xdr:row>48</xdr:row>
+      <xdr:rowOff>56029</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="직사각형 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E100FA21-BB77-3B60-6C37-BBF7FCC9749A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1277471" y="9076765"/>
+          <a:ext cx="1541555" cy="1098176"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="57150">
+          <a:solidFill>
+            <a:srgbClr val="FF0000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="ko-KR" altLang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>257735</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>56029</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>44824</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>112059</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="5" name="별: 꼭짓점 5개 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EB8FAFA2-D775-9F8F-9485-79552DE04892}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1042147" y="8561294"/>
+          <a:ext cx="392206" cy="459441"/>
+        </a:xfrm>
+        <a:prstGeom prst="star5">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFF00"/>
+        </a:solidFill>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="15000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:endParaRPr lang="ko-KR" altLang="en-US" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>7</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>30</xdr:col>
+      <xdr:colOff>500700</xdr:colOff>
+      <xdr:row>47</xdr:row>
+      <xdr:rowOff>70410</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="20" name="그림 19">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1FB2449D-C0F2-41F9-966E-C658CEBA3174}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3810000" y="8303559"/>
+          <a:ext cx="14418406" cy="1684057"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 테마">
   <a:themeElements>
@@ -1660,93 +4317,93 @@
   <sheetData>
     <row r="1" spans="2:15" ht="16.5" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="2" spans="2:15" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B2" s="43" t="s">
+      <c r="B2" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="38" t="s">
+      <c r="C2" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="36" t="s">
+      <c r="D2" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="36" t="s">
+      <c r="E2" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="37" t="s">
+      <c r="F2" s="26" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="3" spans="2:15" ht="53" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B3" s="44" t="s">
+      <c r="B3" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="39" t="s">
+      <c r="C3" s="28" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="33" t="s">
+      <c r="D3" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="34" t="s">
+      <c r="E3" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="F3" s="35"/>
+      <c r="F3" s="24"/>
     </row>
     <row r="4" spans="2:15" ht="143" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B4" s="45" t="s">
+      <c r="B4" s="34" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="40" t="s">
+      <c r="C4" s="29" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E4" s="19" t="s">
+      <c r="E4" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="F4" s="28"/>
+      <c r="F4" s="20"/>
     </row>
     <row r="5" spans="2:15" ht="83" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B5" s="45" t="s">
+      <c r="B5" s="34" t="s">
         <v>26</v>
       </c>
-      <c r="C5" s="41" t="s">
+      <c r="C5" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="D5" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="E5" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="F5" s="28"/>
+      <c r="F5" s="20"/>
     </row>
     <row r="6" spans="2:15" ht="96" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B6" s="45" t="s">
+      <c r="B6" s="34" t="s">
         <v>25</v>
       </c>
-      <c r="C6" s="41" t="s">
+      <c r="C6" s="30" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="E6" s="11" t="s">
+      <c r="E6" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="F6" s="28"/>
+      <c r="F6" s="20"/>
     </row>
     <row r="7" spans="2:15" ht="80" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B7" s="46" t="s">
+      <c r="B7" s="35" t="s">
         <v>28</v>
       </c>
-      <c r="C7" s="42" t="s">
+      <c r="C7" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="D7" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="E7" s="18" t="s">
+      <c r="E7" s="17" t="s">
         <v>30</v>
       </c>
       <c r="F7" s="2"/>
@@ -1796,78 +4453,78 @@
   <sheetData>
     <row r="1" spans="2:15" ht="16.5" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="2" spans="2:15" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B2" s="43" t="s">
+      <c r="B2" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="38" t="s">
+      <c r="C2" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="36" t="s">
+      <c r="D2" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="36" t="s">
+      <c r="E2" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="37" t="s">
+      <c r="F2" s="26" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="3" spans="2:15" ht="53" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B3" s="44" t="s">
+      <c r="B3" s="33" t="s">
         <v>33</v>
       </c>
-      <c r="C3" s="48" t="s">
+      <c r="C3" s="37" t="s">
         <v>49</v>
       </c>
-      <c r="D3" s="33" t="s">
+      <c r="D3" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="E3" s="34" t="s">
+      <c r="E3" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="F3" s="35"/>
+      <c r="F3" s="24"/>
     </row>
     <row r="4" spans="2:15" ht="80" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B4" s="45" t="s">
+      <c r="B4" s="34" t="s">
         <v>37</v>
       </c>
-      <c r="C4" s="40" t="s">
+      <c r="C4" s="29" t="s">
         <v>50</v>
       </c>
-      <c r="D4" s="10" t="s">
+      <c r="D4" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E4" s="19" t="s">
+      <c r="E4" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="F4" s="28"/>
+      <c r="F4" s="20"/>
     </row>
     <row r="5" spans="2:15" ht="35" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="B5" s="45" t="s">
+      <c r="B5" s="34" t="s">
         <v>38</v>
       </c>
-      <c r="C5" s="41" t="s">
+      <c r="C5" s="30" t="s">
         <v>51</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="D5" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E5" s="19" t="s">
+      <c r="E5" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="F5" s="28"/>
+      <c r="F5" s="20"/>
     </row>
     <row r="6" spans="2:15" ht="60" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B6" s="46" t="s">
+      <c r="B6" s="35" t="s">
         <v>48</v>
       </c>
-      <c r="C6" s="42" t="s">
+      <c r="C6" s="31" t="s">
         <v>52</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="D6" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="E6" s="47" t="s">
+      <c r="E6" s="36" t="s">
         <v>53</v>
       </c>
       <c r="F6" s="2"/>
@@ -1896,26 +4553,1542 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4F2116CE-AA76-4C27-91A4-F9FAE5EE8EE5}">
-  <dimension ref="A1"/>
+  <dimension ref="B1:V31"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="16" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="2.81640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="24.453125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="34.36328125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="11.08984375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="29.1796875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="21.81640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="5.26953125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="15.6328125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="17.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="9.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="13" width="10.1796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="9.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.1796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="21" width="10.1796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="18.453125" style="1" customWidth="1"/>
+    <col min="23" max="16384" width="8.7265625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:22" ht="16.5" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="2" spans="2:22" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B2" s="82" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="83" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="84" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" s="84" t="s">
+        <v>0</v>
+      </c>
+      <c r="F2" s="85" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" s="32" t="s">
+        <v>61</v>
+      </c>
+      <c r="I2" s="27" t="s">
+        <v>86</v>
+      </c>
+      <c r="J2" s="25" t="s">
+        <v>87</v>
+      </c>
+      <c r="K2" s="25" t="s">
+        <v>71</v>
+      </c>
+      <c r="L2" s="25" t="s">
+        <v>72</v>
+      </c>
+      <c r="M2" s="25" t="s">
+        <v>73</v>
+      </c>
+      <c r="N2" s="25" t="s">
+        <v>74</v>
+      </c>
+      <c r="O2" s="25" t="s">
+        <v>75</v>
+      </c>
+      <c r="P2" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="Q2" s="25" t="s">
+        <v>77</v>
+      </c>
+      <c r="R2" s="25" t="s">
+        <v>78</v>
+      </c>
+      <c r="S2" s="25" t="s">
+        <v>79</v>
+      </c>
+      <c r="T2" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="U2" s="53" t="s">
+        <v>81</v>
+      </c>
+      <c r="V2" s="32" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="3" spans="2:22" ht="53" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B3" s="88" t="s">
+        <v>92</v>
+      </c>
+      <c r="C3" s="87" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3" s="65" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" s="86" t="s">
+        <v>53</v>
+      </c>
+      <c r="F3" s="66"/>
+      <c r="H3" s="54" t="s">
+        <v>62</v>
+      </c>
+      <c r="I3" s="55">
+        <v>34.112000000000002</v>
+      </c>
+      <c r="J3" s="56">
+        <v>3.9236629999999999</v>
+      </c>
+      <c r="K3" s="56">
+        <v>3.7578459999999998</v>
+      </c>
+      <c r="L3" s="56">
+        <v>3.9521470000000001</v>
+      </c>
+      <c r="M3" s="56">
+        <v>4.0604880000000003</v>
+      </c>
+      <c r="N3" s="56">
+        <v>3.8377029999999999</v>
+      </c>
+      <c r="O3" s="56">
+        <v>4.0813430000000004</v>
+      </c>
+      <c r="P3" s="56">
+        <v>4.0691350000000002</v>
+      </c>
+      <c r="Q3" s="56">
+        <v>4.0253920000000001</v>
+      </c>
+      <c r="R3" s="56">
+        <v>3.9643549999999999</v>
+      </c>
+      <c r="S3" s="56">
+        <v>4.0172530000000002</v>
+      </c>
+      <c r="T3" s="56">
+        <v>4.0528579999999996</v>
+      </c>
+      <c r="U3" s="57">
+        <v>3.892128</v>
+      </c>
+      <c r="V3" s="92" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="4" spans="2:22" ht="80" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B4" s="63" t="s">
+        <v>93</v>
+      </c>
+      <c r="C4" s="29" t="s">
+        <v>50</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="E4" s="18" t="s">
+        <v>53</v>
+      </c>
+      <c r="F4" s="20"/>
+      <c r="H4" s="52" t="s">
+        <v>63</v>
+      </c>
+      <c r="I4" s="46">
+        <v>34.113</v>
+      </c>
+      <c r="J4" s="47">
+        <v>3.9277329999999999</v>
+      </c>
+      <c r="K4" s="47">
+        <v>3.7573379999999998</v>
+      </c>
+      <c r="L4" s="47">
+        <v>3.950113</v>
+      </c>
+      <c r="M4" s="47">
+        <v>4.0625229999999997</v>
+      </c>
+      <c r="N4" s="47">
+        <v>3.8397380000000001</v>
+      </c>
+      <c r="O4" s="47">
+        <v>4.0828689999999996</v>
+      </c>
+      <c r="P4" s="47">
+        <v>4.0706610000000003</v>
+      </c>
+      <c r="Q4" s="47">
+        <v>4.0264090000000001</v>
+      </c>
+      <c r="R4" s="47">
+        <v>3.9674070000000001</v>
+      </c>
+      <c r="S4" s="47">
+        <v>4.0203059999999997</v>
+      </c>
+      <c r="T4" s="47">
+        <v>4.0533669999999997</v>
+      </c>
+      <c r="U4" s="48">
+        <v>3.8916189999999999</v>
+      </c>
+      <c r="V4" s="93"/>
+    </row>
+    <row r="5" spans="2:22" ht="95" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B5" s="81" t="s">
+        <v>94</v>
+      </c>
+      <c r="C5" s="89" t="s">
+        <v>52</v>
+      </c>
+      <c r="D5" s="78" t="s">
+        <v>85</v>
+      </c>
+      <c r="E5" s="90" t="s">
+        <v>133</v>
+      </c>
+      <c r="F5" s="79"/>
+      <c r="H5" s="52" t="s">
+        <v>64</v>
+      </c>
+      <c r="I5" s="46">
+        <v>34.109000000000002</v>
+      </c>
+      <c r="J5" s="47">
+        <v>3.924172</v>
+      </c>
+      <c r="K5" s="47">
+        <v>3.7568290000000002</v>
+      </c>
+      <c r="L5" s="47">
+        <v>3.9521470000000001</v>
+      </c>
+      <c r="M5" s="47">
+        <v>4.0584540000000002</v>
+      </c>
+      <c r="N5" s="47">
+        <v>3.8412639999999998</v>
+      </c>
+      <c r="O5" s="47">
+        <v>4.0808340000000003</v>
+      </c>
+      <c r="P5" s="47">
+        <v>4.0716780000000004</v>
+      </c>
+      <c r="Q5" s="47">
+        <v>4.0259</v>
+      </c>
+      <c r="R5" s="47">
+        <v>3.9638460000000002</v>
+      </c>
+      <c r="S5" s="47">
+        <v>4.0177620000000003</v>
+      </c>
+      <c r="T5" s="47">
+        <v>4.0518409999999996</v>
+      </c>
+      <c r="U5" s="48">
+        <v>3.892636</v>
+      </c>
+      <c r="V5" s="93"/>
+    </row>
+    <row r="6" spans="2:22" ht="19" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B6" s="91" t="s">
+        <v>127</v>
+      </c>
+      <c r="C6" s="98" t="s">
+        <v>132</v>
+      </c>
+      <c r="D6" s="101" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="107" t="s">
+        <v>53</v>
+      </c>
+      <c r="F6" s="104"/>
+      <c r="H6" s="52" t="s">
+        <v>65</v>
+      </c>
+      <c r="I6" s="46">
+        <v>34.095999999999997</v>
+      </c>
+      <c r="J6" s="47">
+        <v>3.924172</v>
+      </c>
+      <c r="K6" s="47">
+        <v>3.7573379999999998</v>
+      </c>
+      <c r="L6" s="47">
+        <v>3.95113</v>
+      </c>
+      <c r="M6" s="47">
+        <v>4.0620139999999996</v>
+      </c>
+      <c r="N6" s="47">
+        <v>3.839229</v>
+      </c>
+      <c r="O6" s="47">
+        <v>4.0803250000000002</v>
+      </c>
+      <c r="P6" s="47">
+        <v>4.0711700000000004</v>
+      </c>
+      <c r="Q6" s="47">
+        <v>4.024883</v>
+      </c>
+      <c r="R6" s="47">
+        <v>3.9638460000000002</v>
+      </c>
+      <c r="S6" s="47">
+        <v>4.0152190000000001</v>
+      </c>
+      <c r="T6" s="47">
+        <v>4.0518409999999996</v>
+      </c>
+      <c r="U6" s="48">
+        <v>3.8951799999999999</v>
+      </c>
+      <c r="V6" s="93"/>
+    </row>
+    <row r="7" spans="2:22" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B7" s="34" t="s">
+        <v>128</v>
+      </c>
+      <c r="C7" s="99"/>
+      <c r="D7" s="102"/>
+      <c r="E7" s="108"/>
+      <c r="F7" s="105"/>
+      <c r="H7" s="58" t="s">
+        <v>66</v>
+      </c>
+      <c r="I7" s="49">
+        <v>34.112000000000002</v>
+      </c>
+      <c r="J7" s="50">
+        <v>3.9236629999999999</v>
+      </c>
+      <c r="K7" s="50">
+        <v>3.7573379999999998</v>
+      </c>
+      <c r="L7" s="50">
+        <v>3.9521470000000001</v>
+      </c>
+      <c r="M7" s="50">
+        <v>4.0615050000000004</v>
+      </c>
+      <c r="N7" s="50">
+        <v>3.8387199999999999</v>
+      </c>
+      <c r="O7" s="50">
+        <v>4.0813430000000004</v>
+      </c>
+      <c r="P7" s="50">
+        <v>4.0691350000000002</v>
+      </c>
+      <c r="Q7" s="50">
+        <v>4.0243739999999999</v>
+      </c>
+      <c r="R7" s="50">
+        <v>3.9648639999999999</v>
+      </c>
+      <c r="S7" s="50">
+        <v>4.0172530000000002</v>
+      </c>
+      <c r="T7" s="50">
+        <v>4.0513320000000004</v>
+      </c>
+      <c r="U7" s="51">
+        <v>3.892636</v>
+      </c>
+      <c r="V7" s="94"/>
+    </row>
+    <row r="8" spans="2:22" ht="19" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B8" s="34" t="s">
+        <v>129</v>
+      </c>
+      <c r="C8" s="99"/>
+      <c r="D8" s="102"/>
+      <c r="E8" s="108"/>
+      <c r="F8" s="105"/>
+      <c r="H8" s="59" t="s">
+        <v>88</v>
+      </c>
+      <c r="I8" s="60">
+        <f>(I4-I$3)/I$3</f>
+        <v>2.9315196998055506E-5</v>
+      </c>
+      <c r="J8" s="60">
+        <f t="shared" ref="J8:U8" si="0">(J4-J$3)/J$3</f>
+        <v>1.037296016502951E-3</v>
+      </c>
+      <c r="K8" s="60">
+        <f t="shared" si="0"/>
+        <v>-1.3518382605352987E-4</v>
+      </c>
+      <c r="L8" s="60">
+        <f t="shared" si="0"/>
+        <v>-5.1465696999633147E-4</v>
+      </c>
+      <c r="M8" s="60">
+        <f t="shared" si="0"/>
+        <v>5.011712877859367E-4</v>
+      </c>
+      <c r="N8" s="60">
+        <f t="shared" si="0"/>
+        <v>5.3026510910308359E-4</v>
+      </c>
+      <c r="O8" s="60">
+        <f t="shared" si="0"/>
+        <v>3.7389653356732089E-4</v>
+      </c>
+      <c r="P8" s="60">
+        <f t="shared" si="0"/>
+        <v>3.7501827784041037E-4</v>
+      </c>
+      <c r="Q8" s="60">
+        <f t="shared" si="0"/>
+        <v>2.5264620191028491E-4</v>
+      </c>
+      <c r="R8" s="60">
+        <f t="shared" si="0"/>
+        <v>7.6986041865581588E-4</v>
+      </c>
+      <c r="S8" s="60">
+        <f t="shared" si="0"/>
+        <v>7.5997205055283506E-4</v>
+      </c>
+      <c r="T8" s="60">
+        <f t="shared" si="0"/>
+        <v>1.2559038584625783E-4</v>
+      </c>
+      <c r="U8" s="60">
+        <f t="shared" si="0"/>
+        <v>-1.3077678843041461E-4</v>
+      </c>
+      <c r="V8" s="95" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="9" spans="2:22" ht="19" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B9" s="35" t="s">
+        <v>131</v>
+      </c>
+      <c r="C9" s="100"/>
+      <c r="D9" s="103"/>
+      <c r="E9" s="109"/>
+      <c r="F9" s="106"/>
+      <c r="H9" s="39" t="s">
+        <v>89</v>
+      </c>
+      <c r="I9" s="42">
+        <f t="shared" ref="I9:U9" si="1">(I5-I$3)/I$3</f>
+        <v>-8.7945590994374816E-5</v>
+      </c>
+      <c r="J9" s="42">
+        <f t="shared" si="1"/>
+        <v>1.297257180344216E-4</v>
+      </c>
+      <c r="K9" s="42">
+        <f t="shared" si="1"/>
+        <v>-2.7063376200078489E-4</v>
+      </c>
+      <c r="L9" s="42">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="M9" s="42">
+        <f t="shared" si="1"/>
+        <v>-5.0092501196902716E-4</v>
+      </c>
+      <c r="N9" s="42">
+        <f t="shared" si="1"/>
+        <v>9.2789879779647496E-4</v>
+      </c>
+      <c r="O9" s="42">
+        <f t="shared" si="1"/>
+        <v>-1.2471385031841056E-4</v>
+      </c>
+      <c r="P9" s="42">
+        <f t="shared" si="1"/>
+        <v>6.2494854557545618E-4</v>
+      </c>
+      <c r="Q9" s="42">
+        <f t="shared" si="1"/>
+        <v>1.2619888944976116E-4</v>
+      </c>
+      <c r="R9" s="42">
+        <f t="shared" si="1"/>
+        <v>-1.2839415239040112E-4</v>
+      </c>
+      <c r="S9" s="42">
+        <f t="shared" si="1"/>
+        <v>1.2670349614527456E-4</v>
+      </c>
+      <c r="T9" s="42">
+        <f t="shared" si="1"/>
+        <v>-2.5093403223109363E-4</v>
+      </c>
+      <c r="U9" s="42">
+        <f t="shared" si="1"/>
+        <v>1.3051985957295158E-4</v>
+      </c>
+      <c r="V9" s="96"/>
+    </row>
+    <row r="10" spans="2:22" x14ac:dyDescent="0.45">
+      <c r="H10" s="39" t="s">
+        <v>90</v>
+      </c>
+      <c r="I10" s="42">
+        <f t="shared" ref="I10:U10" si="2">(I6-I$3)/I$3</f>
+        <v>-4.6904315197013785E-4</v>
+      </c>
+      <c r="J10" s="42">
+        <f t="shared" si="2"/>
+        <v>1.297257180344216E-4</v>
+      </c>
+      <c r="K10" s="42">
+        <f t="shared" si="2"/>
+        <v>-1.3518382605352987E-4</v>
+      </c>
+      <c r="L10" s="42">
+        <f t="shared" si="2"/>
+        <v>-2.5732848499816573E-4</v>
+      </c>
+      <c r="M10" s="42">
+        <f t="shared" si="2"/>
+        <v>3.7581689688511577E-4</v>
+      </c>
+      <c r="N10" s="42">
+        <f t="shared" si="2"/>
+        <v>3.9763368869350711E-4</v>
+      </c>
+      <c r="O10" s="42">
+        <f t="shared" si="2"/>
+        <v>-2.4942770063682111E-4</v>
+      </c>
+      <c r="P10" s="42">
+        <f t="shared" si="2"/>
+        <v>5.0010628794577492E-4</v>
+      </c>
+      <c r="Q10" s="42">
+        <f t="shared" si="2"/>
+        <v>-1.2644731246052378E-4</v>
+      </c>
+      <c r="R10" s="42">
+        <f t="shared" si="2"/>
+        <v>-1.2839415239040112E-4</v>
+      </c>
+      <c r="S10" s="42">
+        <f t="shared" si="2"/>
+        <v>-5.0631613194391568E-4</v>
+      </c>
+      <c r="T10" s="42">
+        <f t="shared" si="2"/>
+        <v>-2.5093403223109363E-4</v>
+      </c>
+      <c r="U10" s="42">
+        <f t="shared" si="2"/>
+        <v>7.8414687286744748E-4</v>
+      </c>
+      <c r="V10" s="96"/>
+    </row>
+    <row r="11" spans="2:22" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="H11" s="61" t="s">
+        <v>91</v>
+      </c>
+      <c r="I11" s="62">
+        <f t="shared" ref="I11:U11" si="3">(I7-I$3)/I$3</f>
+        <v>0</v>
+      </c>
+      <c r="J11" s="62">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="K11" s="62">
+        <f t="shared" si="3"/>
+        <v>-1.3518382605352987E-4</v>
+      </c>
+      <c r="L11" s="62">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="M11" s="62">
+        <f t="shared" si="3"/>
+        <v>2.5046250598451358E-4</v>
+      </c>
+      <c r="N11" s="62">
+        <f t="shared" si="3"/>
+        <v>2.6500226828393068E-4</v>
+      </c>
+      <c r="O11" s="62">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="P11" s="62">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="Q11" s="62">
+        <f t="shared" si="3"/>
+        <v>-2.5289462492104756E-4</v>
+      </c>
+      <c r="R11" s="62">
+        <f t="shared" si="3"/>
+        <v>1.2839415239051315E-4</v>
+      </c>
+      <c r="S11" s="62">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="T11" s="62">
+        <f t="shared" si="3"/>
+        <v>-3.7652441807713231E-4</v>
+      </c>
+      <c r="U11" s="62">
+        <f t="shared" si="3"/>
+        <v>1.3051985957295158E-4</v>
+      </c>
+      <c r="V11" s="97"/>
+    </row>
+    <row r="12" spans="2:22" x14ac:dyDescent="0.45">
+      <c r="H12" s="41" t="s">
+        <v>67</v>
+      </c>
+      <c r="I12" s="43">
+        <v>34.49</v>
+      </c>
+      <c r="J12" s="44">
+        <v>4.0472640000000002</v>
+      </c>
+      <c r="K12" s="44">
+        <v>3.954691</v>
+      </c>
+      <c r="L12" s="44">
+        <v>3.8916189999999999</v>
+      </c>
+      <c r="M12" s="44">
+        <v>3.9887700000000001</v>
+      </c>
+      <c r="N12" s="44">
+        <v>3.8860239999999999</v>
+      </c>
+      <c r="O12" s="44">
+        <v>3.9852089999999998</v>
+      </c>
+      <c r="P12" s="44">
+        <v>4.0793080000000002</v>
+      </c>
+      <c r="Q12" s="44">
+        <v>3.9328189999999998</v>
+      </c>
+      <c r="R12" s="44">
+        <v>3.9516390000000001</v>
+      </c>
+      <c r="S12" s="44">
+        <v>3.9002659999999998</v>
+      </c>
+      <c r="T12" s="44">
+        <v>3.9857179999999999</v>
+      </c>
+      <c r="U12" s="45">
+        <v>3.9119649999999999</v>
+      </c>
+      <c r="V12" s="41"/>
+    </row>
+    <row r="13" spans="2:22" x14ac:dyDescent="0.45">
+      <c r="H13" s="38" t="s">
+        <v>68</v>
+      </c>
+      <c r="I13" s="46">
+        <v>34.347999999999999</v>
+      </c>
+      <c r="J13" s="47">
+        <v>3.8611</v>
+      </c>
+      <c r="K13" s="47">
+        <v>3.912982</v>
+      </c>
+      <c r="L13" s="47">
+        <v>3.8702559999999999</v>
+      </c>
+      <c r="M13" s="47">
+        <v>3.8900929999999998</v>
+      </c>
+      <c r="N13" s="47">
+        <v>4.0426859999999998</v>
+      </c>
+      <c r="O13" s="47">
+        <v>3.7990460000000001</v>
+      </c>
+      <c r="P13" s="47">
+        <v>3.8361770000000002</v>
+      </c>
+      <c r="Q13" s="47">
+        <v>3.892636</v>
+      </c>
+      <c r="R13" s="47">
+        <v>4.055402</v>
+      </c>
+      <c r="S13" s="47">
+        <v>3.9587599999999998</v>
+      </c>
+      <c r="T13" s="47">
+        <v>3.9618120000000001</v>
+      </c>
+      <c r="U13" s="48">
+        <v>4.0025029999999999</v>
+      </c>
+      <c r="V13" s="38"/>
+    </row>
+    <row r="14" spans="2:22" x14ac:dyDescent="0.45">
+      <c r="H14" s="38" t="s">
+        <v>69</v>
+      </c>
+      <c r="I14" s="46">
+        <v>34.856999999999999</v>
+      </c>
+      <c r="J14" s="47">
+        <v>4.132206</v>
+      </c>
+      <c r="K14" s="47">
+        <v>4.0014859999999999</v>
+      </c>
+      <c r="L14" s="47">
+        <v>3.9485869999999998</v>
+      </c>
+      <c r="M14" s="47">
+        <v>3.9206120000000002</v>
+      </c>
+      <c r="N14" s="47">
+        <v>4.0589620000000002</v>
+      </c>
+      <c r="O14" s="47">
+        <v>3.9277329999999999</v>
+      </c>
+      <c r="P14" s="47">
+        <v>3.9043350000000001</v>
+      </c>
+      <c r="Q14" s="47">
+        <v>3.8478759999999999</v>
+      </c>
+      <c r="R14" s="47">
+        <v>3.9521470000000001</v>
+      </c>
+      <c r="S14" s="47">
+        <v>3.924172</v>
+      </c>
+      <c r="T14" s="47">
+        <v>4.0208139999999997</v>
+      </c>
+      <c r="U14" s="48">
+        <v>3.9836830000000001</v>
+      </c>
+      <c r="V14" s="38"/>
+    </row>
+    <row r="15" spans="2:22" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="H15" s="40" t="s">
+        <v>70</v>
+      </c>
+      <c r="I15" s="49">
+        <v>34.036000000000001</v>
+      </c>
+      <c r="J15" s="50">
+        <v>3.9262069999999998</v>
+      </c>
+      <c r="K15" s="50">
+        <v>4.0279350000000003</v>
+      </c>
+      <c r="L15" s="50">
+        <v>4.0498070000000004</v>
+      </c>
+      <c r="M15" s="50">
+        <v>4.013185</v>
+      </c>
+      <c r="N15" s="50">
+        <v>3.965881</v>
+      </c>
+      <c r="O15" s="50">
+        <v>3.965881</v>
+      </c>
+      <c r="P15" s="50">
+        <v>3.8692389999999999</v>
+      </c>
+      <c r="Q15" s="50">
+        <v>3.855505</v>
+      </c>
+      <c r="R15" s="50">
+        <v>3.9145080000000001</v>
+      </c>
+      <c r="S15" s="50">
+        <v>4.0457380000000001</v>
+      </c>
+      <c r="T15" s="50">
+        <v>4.1505179999999999</v>
+      </c>
+      <c r="U15" s="51">
+        <v>4.0640489999999998</v>
+      </c>
+      <c r="V15" s="40"/>
+    </row>
+    <row r="31" spans="16:16" x14ac:dyDescent="0.45">
+      <c r="P31" s="3"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="V3:V7"/>
+    <mergeCell ref="V8:V11"/>
+    <mergeCell ref="C6:C9"/>
+    <mergeCell ref="D6:D9"/>
+    <mergeCell ref="F6:F9"/>
+    <mergeCell ref="E6:E9"/>
+  </mergeCells>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <dataValidations disablePrompts="1" count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D14:D15" xr:uid="{79E234A5-FEEA-4808-9653-9CEFC2710DC3}">
+      <formula1>"O, X"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E4E8E20-17D3-4D94-8621-CB472F24DDEF}">
+  <dimension ref="B1:M11"/>
+  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="16" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="2.81640625" style="1" customWidth="1"/>
+    <col min="2" max="2" width="24.453125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="34.36328125" style="1" customWidth="1"/>
+    <col min="4" max="4" width="11.08984375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="29.1796875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="21.81640625" style="1" customWidth="1"/>
+    <col min="7" max="7" width="5.26953125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="15.6328125" style="1" customWidth="1"/>
+    <col min="9" max="9" width="17.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.54296875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="9.54296875" style="1" customWidth="1"/>
+    <col min="12" max="12" width="10.1796875" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="23.81640625" style="1" customWidth="1"/>
+    <col min="14" max="16384" width="8.7265625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="2" spans="2:13" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B2" s="82" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" s="83" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="84" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" s="84" t="s">
+        <v>0</v>
+      </c>
+      <c r="F2" s="85" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" s="32" t="s">
+        <v>137</v>
+      </c>
+      <c r="I2" s="27" t="s">
+        <v>86</v>
+      </c>
+      <c r="J2" s="25" t="s">
+        <v>139</v>
+      </c>
+      <c r="K2" s="25" t="s">
+        <v>87</v>
+      </c>
+      <c r="L2" s="53" t="s">
+        <v>71</v>
+      </c>
+      <c r="M2" s="32" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="3" spans="2:13" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B3" s="88" t="s">
+        <v>136</v>
+      </c>
+      <c r="C3" s="87" t="s">
+        <v>140</v>
+      </c>
+      <c r="D3" s="65"/>
+      <c r="E3" s="86" t="s">
+        <v>53</v>
+      </c>
+      <c r="F3" s="66"/>
+      <c r="H3" s="136" t="s">
+        <v>138</v>
+      </c>
+      <c r="I3" s="43">
+        <v>49.133000000000003</v>
+      </c>
+      <c r="J3" s="44">
+        <v>1.47956</v>
+      </c>
+      <c r="K3" s="44">
+        <v>4.2858169999999998</v>
+      </c>
+      <c r="L3" s="45">
+        <v>4.3768630000000002</v>
+      </c>
+      <c r="M3" s="135"/>
+    </row>
+    <row r="4" spans="2:13" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="B4" s="63"/>
+      <c r="C4" s="29"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="18"/>
+      <c r="F4" s="20"/>
+      <c r="H4" s="52" t="s">
+        <v>67</v>
+      </c>
+      <c r="I4" s="46">
+        <v>49.155999999999999</v>
+      </c>
+      <c r="J4" s="47">
+        <v>1.481978</v>
+      </c>
+      <c r="K4" s="47">
+        <v>4.237495</v>
+      </c>
+      <c r="L4" s="48">
+        <v>4.3315939999999999</v>
+      </c>
+      <c r="M4" s="129"/>
+    </row>
+    <row r="5" spans="2:13" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B5" s="152"/>
+      <c r="C5" s="31"/>
+      <c r="D5" s="17"/>
+      <c r="E5" s="36"/>
+      <c r="F5" s="2"/>
+      <c r="H5" s="52" t="s">
+        <v>68</v>
+      </c>
+      <c r="I5" s="46">
+        <v>49.137</v>
+      </c>
+      <c r="J5" s="47">
+        <v>1.4811719999999999</v>
+      </c>
+      <c r="K5" s="47">
+        <v>4.2675049999999999</v>
+      </c>
+      <c r="L5" s="48">
+        <v>4.3656730000000001</v>
+      </c>
+      <c r="M5" s="129"/>
+    </row>
+    <row r="6" spans="2:13" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="H6" s="131" t="s">
+        <v>69</v>
+      </c>
+      <c r="I6" s="132">
+        <v>49.177999999999997</v>
+      </c>
+      <c r="J6" s="133">
+        <v>1.478755</v>
+      </c>
+      <c r="K6" s="133">
+        <v>4.2624190000000004</v>
+      </c>
+      <c r="L6" s="137">
+        <v>4.3524479999999999</v>
+      </c>
+      <c r="M6" s="134"/>
+    </row>
+    <row r="7" spans="2:13" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="H7" s="139" t="s">
+        <v>141</v>
+      </c>
+      <c r="I7" s="140">
+        <f>AVERAGE(I3:I6)</f>
+        <v>49.150999999999996</v>
+      </c>
+      <c r="J7" s="141">
+        <f t="shared" ref="J7:L7" si="0">AVERAGE(J3:J6)</f>
+        <v>1.4803662499999999</v>
+      </c>
+      <c r="K7" s="141">
+        <f t="shared" si="0"/>
+        <v>4.2633090000000005</v>
+      </c>
+      <c r="L7" s="142">
+        <f t="shared" si="0"/>
+        <v>4.3566444999999998</v>
+      </c>
+      <c r="M7" s="139"/>
+    </row>
+    <row r="8" spans="2:13" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="H8" s="138" t="s">
+        <v>143</v>
+      </c>
+      <c r="I8" s="143">
+        <f>(I3-I$7)/I$7</f>
+        <v>-3.6621838823205178E-4</v>
+      </c>
+      <c r="J8" s="144">
+        <f t="shared" ref="J8:L8" si="1">(J3-J$7)/J$7</f>
+        <v>-5.4462873630082924E-4</v>
+      </c>
+      <c r="K8" s="144">
+        <f t="shared" si="1"/>
+        <v>5.2794671932058649E-3</v>
+      </c>
+      <c r="L8" s="145">
+        <f t="shared" si="1"/>
+        <v>4.6408422812557609E-3</v>
+      </c>
+      <c r="M8" s="130" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="9" spans="2:13" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="H9" s="39" t="s">
+        <v>144</v>
+      </c>
+      <c r="I9" s="146">
+        <f t="shared" ref="I9:L9" si="2">(I4-I$7)/I$7</f>
+        <v>1.0172733006454718E-4</v>
+      </c>
+      <c r="J9" s="147">
+        <f t="shared" si="2"/>
+        <v>1.088750841219282E-3</v>
+      </c>
+      <c r="K9" s="147">
+        <f t="shared" si="2"/>
+        <v>-6.054921189151536E-3</v>
+      </c>
+      <c r="L9" s="148">
+        <f t="shared" si="2"/>
+        <v>-5.7499527445950358E-3</v>
+      </c>
+      <c r="M9" s="96"/>
+    </row>
+    <row r="10" spans="2:13" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="H10" s="39" t="s">
+        <v>145</v>
+      </c>
+      <c r="I10" s="146">
+        <f t="shared" ref="I10:L11" si="3">(I5-I$7)/I$7</f>
+        <v>-2.8483652418050077E-4</v>
+      </c>
+      <c r="J10" s="147">
+        <f t="shared" si="3"/>
+        <v>5.4429098204586163E-4</v>
+      </c>
+      <c r="K10" s="147">
+        <f t="shared" si="3"/>
+        <v>9.8421202873153748E-4</v>
+      </c>
+      <c r="L10" s="148">
+        <f t="shared" si="3"/>
+        <v>2.0723517835803057E-3</v>
+      </c>
+      <c r="M10" s="96"/>
+    </row>
+    <row r="11" spans="2:13" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="H11" s="61" t="s">
+        <v>146</v>
+      </c>
+      <c r="I11" s="149">
+        <f t="shared" si="3"/>
+        <v>5.4932758234829454E-4</v>
+      </c>
+      <c r="J11" s="150">
+        <f t="shared" si="3"/>
+        <v>-1.0884130869640146E-3</v>
+      </c>
+      <c r="K11" s="150">
+        <f t="shared" si="3"/>
+        <v>-2.0875803278628345E-4</v>
+      </c>
+      <c r="L11" s="151">
+        <f t="shared" si="3"/>
+        <v>-9.6324132024082679E-4</v>
+      </c>
+      <c r="M11" s="97"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="M8:M11"/>
+  </mergeCells>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <dataValidations disablePrompts="1" count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D14:D15" xr:uid="{A365DB84-01A0-4E66-B509-ACB4E3A3C22A}">
+      <formula1>"O, X"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34DA6E25-AFEB-42BB-9630-8291C8EB2B20}">
+  <dimension ref="B1:AA39"/>
   <sheetFormatPr defaultRowHeight="16" x14ac:dyDescent="0.45"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="2.6328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:20" ht="16.5" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="2" spans="2:20" ht="26.5" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B2" s="110" t="s">
+        <v>96</v>
+      </c>
+      <c r="C2" s="111"/>
+      <c r="D2" s="111"/>
+      <c r="E2" s="111"/>
+      <c r="F2" s="111"/>
+      <c r="G2" s="111"/>
+      <c r="H2" s="111"/>
+      <c r="I2" s="111"/>
+      <c r="J2" s="112"/>
+      <c r="L2" s="110" t="s">
+        <v>95</v>
+      </c>
+      <c r="M2" s="111"/>
+      <c r="N2" s="111"/>
+      <c r="O2" s="111"/>
+      <c r="P2" s="111"/>
+      <c r="Q2" s="111"/>
+      <c r="R2" s="111"/>
+      <c r="S2" s="111"/>
+      <c r="T2" s="112"/>
+    </row>
+    <row r="25" spans="2:27" ht="16.5" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="26" spans="2:27" ht="26.5" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B26" s="113" t="s">
+        <v>98</v>
+      </c>
+      <c r="C26" s="114"/>
+      <c r="D26" s="114"/>
+      <c r="E26" s="114"/>
+      <c r="F26" s="114"/>
+      <c r="G26" s="115"/>
+      <c r="I26" s="113" t="s">
+        <v>97</v>
+      </c>
+      <c r="J26" s="114"/>
+      <c r="K26" s="114"/>
+      <c r="L26" s="114"/>
+      <c r="M26" s="114"/>
+      <c r="N26" s="114"/>
+      <c r="O26" s="114"/>
+      <c r="P26" s="114"/>
+      <c r="Q26" s="114"/>
+      <c r="R26" s="114"/>
+      <c r="S26" s="114"/>
+      <c r="T26" s="114"/>
+      <c r="U26" s="114"/>
+      <c r="V26" s="114"/>
+      <c r="W26" s="114"/>
+      <c r="X26" s="114"/>
+      <c r="Y26" s="114"/>
+      <c r="Z26" s="114"/>
+      <c r="AA26" s="116"/>
+    </row>
+    <row r="38" spans="2:7" ht="16.5" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="39" spans="2:7" ht="26.5" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B39" s="113" t="s">
+        <v>130</v>
+      </c>
+      <c r="C39" s="114"/>
+      <c r="D39" s="114"/>
+      <c r="E39" s="114"/>
+      <c r="F39" s="114"/>
+      <c r="G39" s="115"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="B2:J2"/>
+    <mergeCell ref="L2:T2"/>
+    <mergeCell ref="B26:G26"/>
+    <mergeCell ref="I26:AA26"/>
+    <mergeCell ref="B39:G39"/>
+  </mergeCells>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C2B1110-480D-43CA-ADDF-C33DF1BCB179}">
+  <dimension ref="B1:H27"/>
+  <sheetFormatPr defaultRowHeight="16" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="2.6328125" customWidth="1"/>
+    <col min="2" max="4" width="26" customWidth="1"/>
+    <col min="6" max="7" width="23.90625" customWidth="1"/>
+    <col min="8" max="8" width="17.36328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="2" spans="2:8" x14ac:dyDescent="0.45">
+      <c r="B2" s="123" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" s="124"/>
+      <c r="D2" s="125"/>
+      <c r="F2" s="119" t="s">
+        <v>31</v>
+      </c>
+      <c r="G2" s="101"/>
+      <c r="H2" s="120"/>
+    </row>
+    <row r="3" spans="2:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B3" s="77" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="78" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="79" t="s">
+        <v>39</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="G3" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="4" spans="2:8" x14ac:dyDescent="0.45">
+      <c r="B4" s="64" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="76" t="s">
+        <v>3</v>
+      </c>
+      <c r="D4" s="80" t="s">
+        <v>54</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="G4" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="H4" s="117" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="2:8" x14ac:dyDescent="0.45">
+      <c r="B5" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="F5" s="14" t="s">
+        <v>44</v>
+      </c>
+      <c r="G5" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="H5" s="118"/>
+    </row>
+    <row r="6" spans="2:8" x14ac:dyDescent="0.45">
+      <c r="B6" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="F6" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="G6" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="H6" s="13" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B7" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="F7" s="121" t="s">
+        <v>41</v>
+      </c>
+      <c r="G7" s="122"/>
+      <c r="H7" s="15" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="2:8" x14ac:dyDescent="0.45">
+      <c r="B8" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="F8" s="11"/>
+      <c r="G8" s="11"/>
+      <c r="H8" s="11"/>
+    </row>
+    <row r="9" spans="2:8" x14ac:dyDescent="0.45">
+      <c r="B9" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="19" t="s">
+        <v>3</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11"/>
+    </row>
+    <row r="10" spans="2:8" x14ac:dyDescent="0.45">
+      <c r="B10" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C10" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="F10" s="11"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="11"/>
+    </row>
+    <row r="11" spans="2:8" x14ac:dyDescent="0.45">
+      <c r="B11" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="F11" s="11"/>
+      <c r="G11" s="11"/>
+      <c r="H11" s="11"/>
+    </row>
+    <row r="12" spans="2:8" x14ac:dyDescent="0.45">
+      <c r="B12" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C12" s="19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="F12" s="11"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="11"/>
+    </row>
+    <row r="13" spans="2:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B13" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="C13" s="21" t="s">
+        <v>124</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="F13" s="11"/>
+      <c r="G13" s="11"/>
+      <c r="H13" s="11"/>
+    </row>
+    <row r="14" spans="2:8" x14ac:dyDescent="0.45">
+      <c r="B14" s="127"/>
+      <c r="C14" s="128"/>
+      <c r="D14" s="128"/>
+      <c r="F14" s="11"/>
+      <c r="G14" s="11"/>
+      <c r="H14" s="11"/>
+    </row>
+    <row r="15" spans="2:8" x14ac:dyDescent="0.45">
+      <c r="H15" s="11"/>
+    </row>
+    <row r="16" spans="2:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.5"/>
+    <row r="17" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B17" s="123" t="s">
+        <v>99</v>
+      </c>
+      <c r="C17" s="124"/>
+      <c r="D17" s="125"/>
+    </row>
+    <row r="18" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B18" s="6" t="s">
+        <v>1</v>
+      </c>
+      <c r="C18" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="19" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B19" s="67" t="s">
+        <v>2</v>
+      </c>
+      <c r="C19" s="68" t="s">
+        <v>3</v>
+      </c>
+      <c r="D19" s="69" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="20" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B20" s="70" t="s">
+        <v>4</v>
+      </c>
+      <c r="C20" s="71" t="s">
+        <v>3</v>
+      </c>
+      <c r="D20" s="72" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="21" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B21" s="70" t="s">
+        <v>5</v>
+      </c>
+      <c r="C21" s="71" t="s">
+        <v>3</v>
+      </c>
+      <c r="D21" s="72" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="22" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B22" s="70" t="s">
+        <v>6</v>
+      </c>
+      <c r="C22" s="71" t="s">
+        <v>3</v>
+      </c>
+      <c r="D22" s="72" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="23" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B23" s="70" t="s">
+        <v>7</v>
+      </c>
+      <c r="C23" s="71" t="s">
+        <v>3</v>
+      </c>
+      <c r="D23" s="72" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="24" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B24" s="70" t="s">
+        <v>8</v>
+      </c>
+      <c r="C24" s="71" t="s">
+        <v>3</v>
+      </c>
+      <c r="D24" s="72" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="25" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B25" s="70" t="s">
+        <v>45</v>
+      </c>
+      <c r="C25" s="71" t="s">
+        <v>9</v>
+      </c>
+      <c r="D25" s="72" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="26" spans="2:4" x14ac:dyDescent="0.45">
+      <c r="B26" s="70" t="s">
+        <v>46</v>
+      </c>
+      <c r="C26" s="71" t="s">
+        <v>9</v>
+      </c>
+      <c r="D26" s="72" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="27" spans="2:4" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B27" s="73" t="s">
+        <v>47</v>
+      </c>
+      <c r="C27" s="74" t="s">
+        <v>10</v>
+      </c>
+      <c r="D27" s="75" t="s">
+        <v>60</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="B17:D17"/>
+  </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{34DA6E25-AFEB-42BB-9630-8291C8EB2B20}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="16" x14ac:dyDescent="0.45"/>
-  <sheetData/>
-  <phoneticPr fontId="2" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C2B1110-480D-43CA-ADDF-C33DF1BCB179}">
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7DFE7FBE-CFE6-404A-8EE0-068E5E4122A1}">
   <dimension ref="B1:H13"/>
   <sheetFormatPr defaultRowHeight="16" x14ac:dyDescent="0.45"/>
   <cols>
@@ -1927,31 +6100,31 @@
   <sheetData>
     <row r="1" spans="2:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.5"/>
     <row r="2" spans="2:8" x14ac:dyDescent="0.45">
-      <c r="B2" s="30" t="s">
-        <v>12</v>
-      </c>
-      <c r="C2" s="31"/>
-      <c r="D2" s="32"/>
-      <c r="F2" s="20" t="s">
-        <v>31</v>
-      </c>
-      <c r="G2" s="24"/>
-      <c r="H2" s="21"/>
+      <c r="B2" s="123" t="s">
+        <v>125</v>
+      </c>
+      <c r="C2" s="124"/>
+      <c r="D2" s="125"/>
+      <c r="F2" s="119" t="s">
+        <v>126</v>
+      </c>
+      <c r="G2" s="101"/>
+      <c r="H2" s="120"/>
     </row>
     <row r="3" spans="2:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="77" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="78" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="79" t="s">
         <v>39</v>
       </c>
       <c r="F3" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="G3" s="18" t="s">
+      <c r="G3" s="17" t="s">
         <v>11</v>
       </c>
       <c r="H3" s="2" t="s">
@@ -1959,160 +6132,160 @@
       </c>
     </row>
     <row r="4" spans="2:8" x14ac:dyDescent="0.45">
-      <c r="B4" s="8" t="s">
-        <v>2</v>
-      </c>
-      <c r="C4" s="17" t="s">
-        <v>3</v>
-      </c>
-      <c r="D4" s="9" t="s">
-        <v>54</v>
-      </c>
-      <c r="F4" s="8" t="s">
+      <c r="B4" s="64" t="s">
+        <v>100</v>
+      </c>
+      <c r="C4" s="76" t="s">
+        <v>101</v>
+      </c>
+      <c r="D4" s="80" t="s">
+        <v>102</v>
+      </c>
+      <c r="F4" s="64" t="s">
         <v>42</v>
       </c>
-      <c r="G4" s="17" t="s">
-        <v>32</v>
-      </c>
-      <c r="H4" s="22" t="s">
+      <c r="G4" s="76" t="s">
+        <v>124</v>
+      </c>
+      <c r="H4" s="126" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B5" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="C5" s="27" t="s">
-        <v>3</v>
+        <v>103</v>
+      </c>
+      <c r="C5" s="19" t="s">
+        <v>104</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="F5" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="F5" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="G5" s="13" t="s">
+      <c r="G5" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="H5" s="23"/>
-    </row>
-    <row r="6" spans="2:8" x14ac:dyDescent="0.45">
+      <c r="H5" s="118"/>
+    </row>
+    <row r="6" spans="2:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
       <c r="B6" s="4" t="s">
-        <v>5</v>
-      </c>
-      <c r="C6" s="27" t="s">
-        <v>3</v>
+        <v>105</v>
+      </c>
+      <c r="C6" s="19" t="s">
+        <v>9</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="F6" s="15" t="s">
-        <v>43</v>
-      </c>
-      <c r="G6" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="H6" s="14" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="7" spans="2:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+        <v>106</v>
+      </c>
+      <c r="F6" s="121" t="s">
+        <v>41</v>
+      </c>
+      <c r="G6" s="122"/>
+      <c r="H6" s="15" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B7" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7" s="27" t="s">
-        <v>3</v>
+        <v>107</v>
+      </c>
+      <c r="C7" s="19" t="s">
+        <v>108</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="F7" s="25" t="s">
-        <v>41</v>
-      </c>
-      <c r="G7" s="26"/>
-      <c r="H7" s="16" t="s">
-        <v>40</v>
+        <v>109</v>
       </c>
     </row>
     <row r="8" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B8" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C8" s="27" t="s">
-        <v>3</v>
+        <v>110</v>
+      </c>
+      <c r="C8" s="19" t="s">
+        <v>9</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="F8" s="12"/>
-      <c r="G8" s="12"/>
-      <c r="H8" s="12"/>
+        <v>113</v>
+      </c>
+      <c r="F8" s="11"/>
+      <c r="G8" s="11"/>
+      <c r="H8" s="11"/>
     </row>
     <row r="9" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B9" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C9" s="27" t="s">
-        <v>3</v>
+        <v>111</v>
+      </c>
+      <c r="C9" s="19" t="s">
+        <v>9</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="F9" s="12"/>
-      <c r="G9" s="12"/>
-      <c r="H9" s="12"/>
+        <v>114</v>
+      </c>
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11"/>
     </row>
     <row r="10" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B10" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="C10" s="27" t="s">
+        <v>112</v>
+      </c>
+      <c r="C10" s="19" t="s">
         <v>9</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="F10" s="12"/>
-      <c r="G10" s="12"/>
-      <c r="H10" s="12"/>
+        <v>115</v>
+      </c>
+      <c r="F10" s="11"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="11"/>
     </row>
     <row r="11" spans="2:8" x14ac:dyDescent="0.45">
       <c r="B11" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="C11" s="27" t="s">
+        <v>116</v>
+      </c>
+      <c r="C11" s="19" t="s">
+        <v>117</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="F11" s="11"/>
+      <c r="G11" s="11"/>
+      <c r="H11" s="11"/>
+    </row>
+    <row r="12" spans="2:8" x14ac:dyDescent="0.45">
+      <c r="B12" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="C12" s="19" t="s">
+        <v>120</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="F12" s="11"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="11"/>
+    </row>
+    <row r="13" spans="2:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
+      <c r="B13" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="C13" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="D11" s="5" t="s">
-        <v>56</v>
-      </c>
-      <c r="F11" s="12"/>
-      <c r="G11" s="12"/>
-      <c r="H11" s="12"/>
-    </row>
-    <row r="12" spans="2:8" ht="16.5" thickBot="1" x14ac:dyDescent="0.5">
-      <c r="B12" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="C12" s="29" t="s">
-        <v>10</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="F12" s="12"/>
-      <c r="G12" s="12"/>
-      <c r="H12" s="12"/>
-    </row>
-    <row r="13" spans="2:8" x14ac:dyDescent="0.45">
-      <c r="H13" s="12"/>
+      <c r="D13" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="H13" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="F2:H2"/>
     <mergeCell ref="H4:H5"/>
-    <mergeCell ref="F2:H2"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="F6:G6"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>